<commit_message>
addded the report connections features in the slicers to apply the slicers in the dashboard to every pivot chart
</commit_message>
<xml_diff>
--- a/Fully_Cleaned_Jumia_Dataset..xlsx
+++ b/Fully_Cleaned_Jumia_Dataset..xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\excel dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{73E9ECA9-E9AA-47FB-B19F-98C7E86575DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB028425-1072-4A54-99F0-F5DD2FE7C97F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DC2EBC4B-1350-4004-B5CD-B48C2EF83F67}"/>
   </bookViews>
@@ -32,8 +32,8 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="18" r:id="rId11"/>
-    <pivotCache cacheId="16" r:id="rId12"/>
+    <pivotCache cacheId="0" r:id="rId11"/>
+    <pivotCache cacheId="1" r:id="rId12"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
@@ -85,7 +85,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="146">
   <si>
     <t>Product</t>
   </si>
@@ -492,9 +492,6 @@
     <t>Sum of Ratingd</t>
   </si>
   <si>
-    <t>(Multiple Items)</t>
-  </si>
-  <si>
     <t>High Discount</t>
   </si>
   <si>
@@ -523,6 +520,9 @@
   </si>
   <si>
     <t>Count of Product</t>
+  </si>
+  <si>
+    <t>(All)</t>
   </si>
 </sst>
 </file>
@@ -1081,11 +1081,11 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="11" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1134,14 +1134,7 @@
   </cellStyles>
   <dxfs count="6">
     <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="14" formatCode="0.00%"/>
@@ -1153,7 +1146,14 @@
       <numFmt numFmtId="14" formatCode="0.00%"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <numFmt numFmtId="14" formatCode="0.00%"/>
@@ -1831,7 +1831,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-KE"/>
+          <a:endParaRPr lang="nl-NL"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -3151,6 +3151,62 @@
           </c:extLst>
         </c:dLbl>
       </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="10"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-KE"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
     </c:pivotFmts>
     <c:plotArea>
       <c:layout/>
@@ -4313,7 +4369,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-KE"/>
+          <a:endParaRPr lang="nl-NL"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -16434,8 +16490,8 @@
       <xdr:row>23</xdr:row>
       <xdr:rowOff>81915</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="13" name="discount category 1">
@@ -16458,7 +16514,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -16512,8 +16568,8 @@
       <xdr:row>23</xdr:row>
       <xdr:rowOff>81915</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="14" name="Review 1">
@@ -16536,7 +16592,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -16590,8 +16646,8 @@
       <xdr:row>37</xdr:row>
       <xdr:rowOff>104775</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="15" name="Rating category 1">
@@ -16614,7 +16670,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -16668,8 +16724,8 @@
       <xdr:row>37</xdr:row>
       <xdr:rowOff>112395</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="16" name="Ratingd 1">
@@ -16692,7 +16748,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -16787,8 +16843,8 @@
       <xdr:row>26</xdr:row>
       <xdr:rowOff>158115</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="3" name="discount category">
@@ -16811,7 +16867,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -16865,8 +16921,8 @@
       <xdr:row>30</xdr:row>
       <xdr:rowOff>74295</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="4" name="Review">
@@ -16889,7 +16945,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -17020,8 +17076,8 @@
       <xdr:row>38</xdr:row>
       <xdr:rowOff>43815</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="5" name="Rating category">
@@ -17044,7 +17100,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -17139,8 +17195,8 @@
       <xdr:row>24</xdr:row>
       <xdr:rowOff>127635</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="3" name="Ratingd">
@@ -17163,7 +17219,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -20302,7 +20358,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B14D74A0-D809-4085-99CB-E4A66B10EE1E}" name="PivotTable6" cacheId="18" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B14D74A0-D809-4085-99CB-E4A66B10EE1E}" name="PivotTable6" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
   <location ref="A3:B11" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField showAll="0"/>
@@ -20354,9 +20410,45 @@
         <item t="default"/>
       </items>
     </pivotField>
+    <pivotField showAll="0">
+      <items count="24">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="4"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField showAll="0">
       <items count="5">
         <item x="0"/>
@@ -20403,7 +20495,7 @@
     <dataField name="Sum of Review" fld="4" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="1">
+    <format dxfId="5">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
@@ -20444,14 +20536,42 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{39DF0057-7429-49A1-88D8-5FDC28DEF6BC}" name="PivotTable7" cacheId="18" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{39DF0057-7429-49A1-88D8-5FDC28DEF6BC}" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11">
   <location ref="A3:B27" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField numFmtId="9" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" showAll="0">
+      <items count="25">
+        <item x="0"/>
+        <item x="11"/>
+        <item x="22"/>
+        <item x="8"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="14"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="1"/>
+        <item x="13"/>
+        <item x="5"/>
+        <item x="7"/>
+        <item x="4"/>
+        <item x="12"/>
+        <item x="20"/>
+        <item x="16"/>
+        <item x="15"/>
+        <item x="21"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="17"/>
+        <item x="6"/>
+        <item x="23"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField axis="axisRow" showAll="0">
       <items count="24">
         <item x="0"/>
@@ -20626,7 +20746,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3069B05E-CF39-4E57-93AD-C7A344F0D354}" name="PivotTable10" cacheId="18" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3069B05E-CF39-4E57-93AD-C7A344F0D354}" name="PivotTable10" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B11" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField axis="axisRow" showAll="0" measureFilter="1">
@@ -20746,7 +20866,35 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField numFmtId="9" showAll="0"/>
-    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="25">
+        <item x="0"/>
+        <item x="11"/>
+        <item x="22"/>
+        <item x="8"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="14"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="1"/>
+        <item x="13"/>
+        <item x="5"/>
+        <item x="7"/>
+        <item x="4"/>
+        <item x="12"/>
+        <item x="20"/>
+        <item x="16"/>
+        <item x="15"/>
+        <item x="21"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="17"/>
+        <item x="6"/>
+        <item x="23"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField dataField="1" showAll="0">
       <items count="24">
         <item x="0"/>
@@ -20776,8 +20924,25 @@
       </items>
     </pivotField>
     <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="4"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
   </pivotFields>
   <rowFields count="1">
     <field x="0"/>
@@ -20836,8 +21001,8 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00AE4C8A-9A64-415E-8E12-CC4796945CF4}" name="PivotTable1" cacheId="18" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2">
-  <location ref="A3:B9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00AE4C8A-9A64-415E-8E12-CC4796945CF4}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2">
+  <location ref="A3:B113" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="9">
     <pivotField axis="axisRow" showAll="0" sortType="ascending">
       <items count="110">
@@ -20965,57 +21130,414 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField numFmtId="9" showAll="0"/>
-    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="25">
+        <item x="0"/>
+        <item x="11"/>
+        <item x="22"/>
+        <item x="8"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="14"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="1"/>
+        <item x="13"/>
+        <item x="5"/>
+        <item x="7"/>
+        <item x="4"/>
+        <item x="12"/>
+        <item x="20"/>
+        <item x="16"/>
+        <item x="15"/>
+        <item x="21"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="17"/>
+        <item x="6"/>
+        <item x="23"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField axis="axisPage" dataField="1" multipleItemSelectionAllowed="1" showAll="0">
       <items count="24">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
-        <item h="1" x="3"/>
-        <item h="1" x="4"/>
-        <item h="1" x="5"/>
-        <item h="1" x="6"/>
-        <item h="1" x="7"/>
-        <item h="1" x="8"/>
-        <item h="1" x="9"/>
-        <item h="1" x="10"/>
-        <item h="1" x="11"/>
-        <item h="1" x="12"/>
-        <item h="1" x="13"/>
-        <item h="1" x="14"/>
-        <item h="1" x="15"/>
-        <item h="1" x="16"/>
-        <item h="1" x="17"/>
-        <item h="1" x="18"/>
-        <item h="1" x="19"/>
-        <item h="1" x="20"/>
-        <item h="1" x="21"/>
-        <item h="1" x="22"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
         <item t="default"/>
       </items>
     </pivotField>
     <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="4"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
   </pivotFields>
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="6">
+  <rowItems count="110">
+    <i>
+      <x v="54"/>
+    </i>
+    <i>
+      <x v="53"/>
+    </i>
+    <i>
+      <x v="46"/>
+    </i>
+    <i>
+      <x v="47"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="48"/>
+    </i>
+    <i>
+      <x v="103"/>
+    </i>
+    <i>
+      <x v="49"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="50"/>
+    </i>
+    <i>
+      <x v="14"/>
+    </i>
+    <i>
+      <x v="51"/>
+    </i>
+    <i>
+      <x v="19"/>
+    </i>
+    <i>
+      <x v="55"/>
+    </i>
+    <i>
+      <x v="23"/>
+    </i>
+    <i>
+      <x v="71"/>
+    </i>
+    <i>
+      <x v="29"/>
+    </i>
+    <i>
+      <x v="74"/>
+    </i>
+    <i>
+      <x v="32"/>
+    </i>
+    <i>
+      <x v="78"/>
+    </i>
+    <i>
+      <x v="34"/>
+    </i>
+    <i>
+      <x v="79"/>
+    </i>
+    <i>
+      <x v="37"/>
+    </i>
+    <i>
+      <x v="81"/>
+    </i>
+    <i>
+      <x v="42"/>
+    </i>
+    <i>
+      <x v="82"/>
+    </i>
+    <i>
+      <x v="45"/>
+    </i>
+    <i>
+      <x v="83"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="85"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="86"/>
+    </i>
+    <i>
+      <x v="21"/>
+    </i>
+    <i>
+      <x v="88"/>
+    </i>
+    <i>
+      <x v="31"/>
+    </i>
+    <i>
+      <x v="89"/>
+    </i>
+    <i>
+      <x v="36"/>
+    </i>
+    <i>
+      <x v="92"/>
+    </i>
+    <i>
+      <x v="43"/>
+    </i>
+    <i>
+      <x v="94"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="96"/>
+    </i>
+    <i>
+      <x v="24"/>
+    </i>
+    <i>
+      <x v="97"/>
+    </i>
+    <i>
+      <x v="39"/>
+    </i>
+    <i>
+      <x v="98"/>
+    </i>
+    <i>
+      <x v="15"/>
+    </i>
+    <i>
+      <x v="99"/>
+    </i>
+    <i>
+      <x v="105"/>
+    </i>
+    <i>
+      <x v="100"/>
+    </i>
+    <i>
+      <x v="33"/>
+    </i>
+    <i>
+      <x v="102"/>
+    </i>
     <i>
       <x v="104"/>
     </i>
     <i>
-      <x v="30"/>
+      <x v="58"/>
     </i>
     <i>
-      <x v="58"/>
+      <x v="30"/>
     </i>
     <i>
       <x v="41"/>
     </i>
     <i>
       <x v="35"/>
+    </i>
+    <i>
+      <x v="106"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i>
+      <x v="25"/>
+    </i>
+    <i>
+      <x v="38"/>
+    </i>
+    <i>
+      <x v="64"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="101"/>
+    </i>
+    <i>
+      <x v="108"/>
+    </i>
+    <i>
+      <x v="84"/>
+    </i>
+    <i>
+      <x v="76"/>
+    </i>
+    <i>
+      <x v="16"/>
+    </i>
+    <i>
+      <x v="66"/>
+    </i>
+    <i>
+      <x v="20"/>
+    </i>
+    <i>
+      <x v="93"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="73"/>
+    </i>
+    <i>
+      <x v="63"/>
+    </i>
+    <i>
+      <x v="56"/>
+    </i>
+    <i>
+      <x v="26"/>
+    </i>
+    <i>
+      <x v="77"/>
+    </i>
+    <i>
+      <x v="62"/>
+    </i>
+    <i>
+      <x v="80"/>
+    </i>
+    <i>
+      <x v="95"/>
+    </i>
+    <i>
+      <x v="67"/>
+    </i>
+    <i>
+      <x v="72"/>
+    </i>
+    <i>
+      <x v="60"/>
+    </i>
+    <i>
+      <x v="61"/>
+    </i>
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="69"/>
+    </i>
+    <i>
+      <x v="27"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="18"/>
+    </i>
+    <i>
+      <x v="75"/>
+    </i>
+    <i>
+      <x v="59"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="91"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="107"/>
+    </i>
+    <i>
+      <x v="28"/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="70"/>
+    </i>
+    <i>
+      <x v="90"/>
+    </i>
+    <i>
+      <x v="22"/>
+    </i>
+    <i>
+      <x v="57"/>
+    </i>
+    <i>
+      <x v="52"/>
+    </i>
+    <i>
+      <x v="40"/>
+    </i>
+    <i>
+      <x v="65"/>
+    </i>
+    <i>
+      <x v="87"/>
+    </i>
+    <i>
+      <x v="44"/>
+    </i>
+    <i>
+      <x v="68"/>
     </i>
     <i t="grand">
       <x/>
@@ -21043,14 +21565,42 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9E40D1CD-3CA5-4738-B295-6EFFD3F2CA97}" name="PivotTable2" cacheId="18" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9E40D1CD-3CA5-4738-B295-6EFFD3F2CA97}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6">
   <location ref="A3:C8" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField numFmtId="9" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" showAll="0">
+      <items count="25">
+        <item x="0"/>
+        <item x="11"/>
+        <item x="22"/>
+        <item x="8"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="14"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="1"/>
+        <item x="13"/>
+        <item x="5"/>
+        <item x="7"/>
+        <item x="4"/>
+        <item x="12"/>
+        <item x="20"/>
+        <item x="16"/>
+        <item x="15"/>
+        <item x="21"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="17"/>
+        <item x="6"/>
+        <item x="23"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField dataField="1" showAll="0">
       <items count="24">
         <item x="0"/>
@@ -21080,7 +21630,16 @@
       </items>
     </pivotField>
     <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="4"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField axis="axisRow" showAll="0">
       <items count="5">
         <item x="0"/>
@@ -21177,7 +21736,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AA63A25A-F0DD-4DA3-A190-10D1E6009A75}" name="PivotTable3" cacheId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AA63A25A-F0DD-4DA3-A190-10D1E6009A75}" name="PivotTable3" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
   <location ref="A3:D14" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField axis="axisRow" showAll="0" measureFilter="1">
@@ -21480,7 +22039,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1C58D286-BDB0-4B94-93B3-6197B5664401}" name="PivotTable4" cacheId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1C58D286-BDB0-4B94-93B3-6197B5664401}" name="PivotTable4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B14" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField axis="axisRow" showAll="0" measureFilter="1">
@@ -21686,7 +22245,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{36F5BBE2-EE30-4DE4-8758-9D8E6E325378}" name="PivotTable5" cacheId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{36F5BBE2-EE30-4DE4-8758-9D8E6E325378}" name="PivotTable5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9">
   <location ref="A3:E8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField dataField="1" showAll="0">
@@ -21995,6 +22554,10 @@
 <slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_discount_category" xr10:uid="{F769AC68-CA91-490A-98F5-0D2D45F20BEE}" sourceName="discount category">
   <pivotTables>
     <pivotTable tabId="5" name="PivotTable6"/>
+    <pivotTable tabId="10" name="PivotTable1"/>
+    <pivotTable tabId="12" name="PivotTable2"/>
+    <pivotTable tabId="9" name="PivotTable10"/>
+    <pivotTable tabId="6" name="PivotTable7"/>
   </pivotTables>
   <data>
     <tabular pivotCacheId="275291811">
@@ -22013,6 +22576,10 @@
 <slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Review" xr10:uid="{46C606D9-82E6-47B6-B9A0-F9DAB9F24664}" sourceName="Review">
   <pivotTables>
     <pivotTable tabId="5" name="PivotTable6"/>
+    <pivotTable tabId="10" name="PivotTable1"/>
+    <pivotTable tabId="12" name="PivotTable2"/>
+    <pivotTable tabId="9" name="PivotTable10"/>
+    <pivotTable tabId="6" name="PivotTable7"/>
   </pivotTables>
   <data>
     <tabular pivotCacheId="275291811">
@@ -22051,6 +22618,10 @@
 <slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Rating_category" xr10:uid="{4F382071-5D20-4766-B821-753F58DAE900}" sourceName="Rating category">
   <pivotTables>
     <pivotTable tabId="6" name="PivotTable7"/>
+    <pivotTable tabId="5" name="PivotTable6"/>
+    <pivotTable tabId="10" name="PivotTable1"/>
+    <pivotTable tabId="12" name="PivotTable2"/>
+    <pivotTable tabId="9" name="PivotTable10"/>
   </pivotTables>
   <data>
     <tabular pivotCacheId="275291811">
@@ -22070,6 +22641,10 @@
 <slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Ratingd" xr10:uid="{0B60ED76-3A5E-4D2F-BE7F-C7B21380BE4D}" sourceName="Ratingd">
   <pivotTables>
     <pivotTable tabId="12" name="PivotTable2"/>
+    <pivotTable tabId="5" name="PivotTable6"/>
+    <pivotTable tabId="10" name="PivotTable1"/>
+    <pivotTable tabId="9" name="PivotTable10"/>
+    <pivotTable tabId="6" name="PivotTable7"/>
   </pivotTables>
   <data>
     <tabular pivotCacheId="275291811">
@@ -22451,12 +23026,12 @@
   <dimension ref="N36:N37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="16384" width="8.88671875" style="16"/>
+    <col min="1" max="16384" width="8.88671875" style="15"/>
   </cols>
   <sheetData>
     <row r="36" spans="14:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="37" spans="14:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="N37" s="17"/>
+      <c r="N37" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -22533,7 +23108,7 @@
         <v>0.64</v>
       </c>
       <c r="G2" s="3">
-        <f>(C2-B2)</f>
+        <f t="shared" ref="G2:G33" si="0">(C2-B2)</f>
         <v>354</v>
       </c>
       <c r="H2" t="str" cm="1">
@@ -22559,7 +23134,7 @@
         <v>0.61</v>
       </c>
       <c r="G3" s="3">
-        <f>(C3-B3)</f>
+        <f t="shared" si="0"/>
         <v>305</v>
       </c>
       <c r="H3" t="str" cm="1">
@@ -22591,7 +23166,7 @@
         <v>2.1</v>
       </c>
       <c r="G4" s="3">
-        <f>(C4-B4)</f>
+        <f t="shared" si="0"/>
         <v>2585</v>
       </c>
       <c r="H4" t="str" cm="1">
@@ -22623,7 +23198,7 @@
         <v>4.8</v>
       </c>
       <c r="G5" s="3">
-        <f>(C5-B5)</f>
+        <f t="shared" si="0"/>
         <v>1526</v>
       </c>
       <c r="H5" t="str" cm="1">
@@ -22649,7 +23224,7 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="G6" s="3">
-        <f>(C6-B6)</f>
+        <f t="shared" si="0"/>
         <v>497</v>
       </c>
       <c r="H6" t="str" cm="1">
@@ -22681,7 +23256,7 @@
         <v>3</v>
       </c>
       <c r="G7" s="3">
-        <f>(C7-B7)</f>
+        <f t="shared" si="0"/>
         <v>528</v>
       </c>
       <c r="H7" t="str" cm="1">
@@ -22713,7 +23288,7 @@
         <v>4.3</v>
       </c>
       <c r="G8" s="3">
-        <f>(C8-B8)</f>
+        <f t="shared" si="0"/>
         <v>2452</v>
       </c>
       <c r="H8" t="str" cm="1">
@@ -22724,8 +23299,8 @@
         <f t="array" ref="I8">_xlfn.IFS(D7&lt;=20%,"Low Disount",D7&lt;=40%,"Medium Discount",D7&gt;40%,"High Discount")</f>
         <v>High Discount</v>
       </c>
-      <c r="K8" s="15"/>
-      <c r="L8" s="15"/>
+      <c r="K8" s="14"/>
+      <c r="L8" s="14"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
@@ -22747,7 +23322,7 @@
         <v>3.3</v>
       </c>
       <c r="G9" s="3">
-        <f>(C9-B9)</f>
+        <f t="shared" si="0"/>
         <v>42</v>
       </c>
       <c r="H9" t="str" cm="1">
@@ -22779,7 +23354,7 @@
         <v>5</v>
       </c>
       <c r="G10" s="3">
-        <f>(C10-B10)</f>
+        <f t="shared" si="0"/>
         <v>189</v>
       </c>
       <c r="H10" t="str" cm="1">
@@ -22811,7 +23386,7 @@
         <v>2.7</v>
       </c>
       <c r="G11" s="3">
-        <f>(C11-B11)</f>
+        <f t="shared" si="0"/>
         <v>355</v>
       </c>
       <c r="H11" t="str" cm="1">
@@ -22843,7 +23418,7 @@
         <v>4.3</v>
       </c>
       <c r="G12" s="3">
-        <f>(C12-B12)</f>
+        <f t="shared" si="0"/>
         <v>197</v>
       </c>
       <c r="H12" t="str" cm="1">
@@ -22875,7 +23450,7 @@
         <v>5</v>
       </c>
       <c r="G13" s="3">
-        <f>(C13-B13)</f>
+        <f t="shared" si="0"/>
         <v>352</v>
       </c>
       <c r="H13" t="str" cm="1">
@@ -22907,7 +23482,7 @@
         <v>2</v>
       </c>
       <c r="G14" s="3">
-        <f>(C14-B14)</f>
+        <f t="shared" si="0"/>
         <v>450</v>
       </c>
       <c r="H14" t="str" cm="1">
@@ -22939,7 +23514,7 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="G15" s="3">
-        <f>(C15-B15)</f>
+        <f t="shared" si="0"/>
         <v>1000</v>
       </c>
       <c r="H15" t="str" cm="1">
@@ -22950,8 +23525,8 @@
         <f t="array" ref="I15">_xlfn.IFS(D14&lt;=20%,"Low Disount",D14&lt;=40%,"Medium Discount",D14&gt;40%,"High Discount")</f>
         <v>High Discount</v>
       </c>
-      <c r="K15" s="14"/>
-      <c r="L15" s="14"/>
+      <c r="K15" s="13"/>
+      <c r="L15" s="13"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
@@ -22967,7 +23542,7 @@
         <v>0.5</v>
       </c>
       <c r="G16" s="3">
-        <f>(C16-B16)</f>
+        <f t="shared" si="0"/>
         <v>1200</v>
       </c>
       <c r="H16" t="str" cm="1">
@@ -22993,7 +23568,7 @@
         <v>0.5</v>
       </c>
       <c r="G17" s="3">
-        <f>(C17-B17)</f>
+        <f t="shared" si="0"/>
         <v>301</v>
       </c>
       <c r="H17" t="str" cm="1">
@@ -23019,7 +23594,7 @@
         <v>0.5</v>
       </c>
       <c r="G18" s="3">
-        <f>(C18-B18)</f>
+        <f t="shared" si="0"/>
         <v>1001</v>
       </c>
       <c r="H18" t="str" cm="1">
@@ -23045,7 +23620,7 @@
         <v>0.5</v>
       </c>
       <c r="G19" s="3">
-        <f>(C19-B19)</f>
+        <f t="shared" si="0"/>
         <v>238</v>
       </c>
       <c r="H19" t="str" cm="1">
@@ -23071,7 +23646,7 @@
         <v>0.5</v>
       </c>
       <c r="G20" s="3">
-        <f>(C20-B20)</f>
+        <f t="shared" si="0"/>
         <v>850</v>
       </c>
       <c r="H20" t="str" cm="1">
@@ -23082,10 +23657,10 @@
         <f t="array" ref="I20">_xlfn.IFS(D19&lt;=20%,"Low Disount",D19&lt;=40%,"Medium Discount",D19&gt;40%,"High Discount")</f>
         <v>High Discount</v>
       </c>
-      <c r="J20" s="14" t="s">
+      <c r="J20" s="13" t="s">
         <v>119</v>
       </c>
-      <c r="K20" s="14">
+      <c r="K20" s="13">
         <f>AVERAGE(C:C)</f>
         <v>1811.1071428571429</v>
       </c>
@@ -23110,7 +23685,7 @@
         <v>2.8</v>
       </c>
       <c r="G21" s="3">
-        <f>(C21-B21)</f>
+        <f t="shared" si="0"/>
         <v>428</v>
       </c>
       <c r="H21" t="str" cm="1">
@@ -23121,10 +23696,10 @@
         <f t="array" ref="I21">_xlfn.IFS(D20&lt;=20%,"Low Disount",D20&lt;=40%,"Medium Discount",D20&gt;40%,"High Discount")</f>
         <v>High Discount</v>
       </c>
-      <c r="J21" s="14" t="s">
+      <c r="J21" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="K21" s="14">
+      <c r="K21" s="13">
         <f>AVERAGE(D:D)</f>
         <v>0.36776785714285737</v>
       </c>
@@ -23150,7 +23725,7 @@
         <v>4</v>
       </c>
       <c r="G22" s="3">
-        <f>(C22-B22)</f>
+        <f t="shared" si="0"/>
         <v>317</v>
       </c>
       <c r="H22" t="str" cm="1">
@@ -23189,7 +23764,7 @@
         <v>4.5999999999999996</v>
       </c>
       <c r="G23" s="3">
-        <f>(C23-B23)</f>
+        <f t="shared" si="0"/>
         <v>968</v>
       </c>
       <c r="H23" t="str" cm="1">
@@ -23200,10 +23775,10 @@
         <f t="array" ref="I23">_xlfn.IFS(D22&lt;=20%,"Low Disount",D22&lt;=40%,"Medium Discount",D22&gt;40%,"High Discount")</f>
         <v>High Discount</v>
       </c>
-      <c r="J23" s="14" t="s">
+      <c r="J23" s="13" t="s">
         <v>119</v>
       </c>
-      <c r="K23" s="14">
+      <c r="K23" s="13">
         <f>AVERAGE(C:C)</f>
         <v>1811.1071428571429</v>
       </c>
@@ -23228,7 +23803,7 @@
         <v>5</v>
       </c>
       <c r="G24" s="3">
-        <f>(C24-B24)</f>
+        <f t="shared" si="0"/>
         <v>941</v>
       </c>
       <c r="H24" t="str" cm="1">
@@ -23239,10 +23814,10 @@
         <f t="array" ref="I24">_xlfn.IFS(D23&lt;=20%,"Low Disount",D23&lt;=40%,"Medium Discount",D23&gt;40%,"High Discount")</f>
         <v>High Discount</v>
       </c>
-      <c r="J24" s="14" t="s">
+      <c r="J24" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="K24" s="14">
+      <c r="K24" s="13">
         <f>AVERAGE(D:D)</f>
         <v>0.36776785714285737</v>
       </c>
@@ -23267,7 +23842,7 @@
         <v>5</v>
       </c>
       <c r="G25" s="3">
-        <f>(C25-B25)</f>
+        <f t="shared" si="0"/>
         <v>1946</v>
       </c>
       <c r="H25" t="str" cm="1">
@@ -23278,10 +23853,10 @@
         <f t="array" ref="I25">_xlfn.IFS(D24&lt;=20%,"Low Disount",D24&lt;=40%,"Medium Discount",D24&gt;40%,"High Discount")</f>
         <v>High Discount</v>
       </c>
-      <c r="J25" s="14" t="s">
+      <c r="J25" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="K25" s="14" t="str">
+      <c r="K25" s="13" t="str">
         <f>_xlfn.XLOOKUP(MIN(B:B), B:B, A:A)</f>
         <v>3PCS Single Head Knitting Crochet Sweater Needle Set</v>
       </c>
@@ -23300,7 +23875,7 @@
         <v>0.49</v>
       </c>
       <c r="G26" s="3">
-        <f>(C26-B26)</f>
+        <f t="shared" si="0"/>
         <v>238</v>
       </c>
       <c r="H26" t="str" cm="1">
@@ -23326,7 +23901,7 @@
         <v>0.49</v>
       </c>
       <c r="G27" s="3">
-        <f>(C27-B27)</f>
+        <f t="shared" si="0"/>
         <v>456</v>
       </c>
       <c r="H27" t="str" cm="1">
@@ -23352,7 +23927,7 @@
         <v>0.49</v>
       </c>
       <c r="G28" s="3">
-        <f>(C28-B28)</f>
+        <f t="shared" si="0"/>
         <v>220</v>
       </c>
       <c r="H28" t="str" cm="1">
@@ -23378,7 +23953,7 @@
         <v>0.49</v>
       </c>
       <c r="G29" s="3">
-        <f>(C29-B29)</f>
+        <f t="shared" si="0"/>
         <v>768</v>
       </c>
       <c r="H29" t="str" cm="1">
@@ -23404,7 +23979,7 @@
         <v>0.49</v>
       </c>
       <c r="G30" s="3">
-        <f>(C30-B30)</f>
+        <f t="shared" si="0"/>
         <v>631</v>
       </c>
       <c r="H30" t="str" cm="1">
@@ -23430,7 +24005,7 @@
         <v>0.49</v>
       </c>
       <c r="G31" s="3">
-        <f>(C31-B31)</f>
+        <f t="shared" si="0"/>
         <v>504</v>
       </c>
       <c r="H31" t="str" cm="1">
@@ -23456,7 +24031,7 @@
         <v>0.49</v>
       </c>
       <c r="G32" s="3">
-        <f>(C32-B32)</f>
+        <f t="shared" si="0"/>
         <v>645</v>
       </c>
       <c r="H32" t="str" cm="1">
@@ -23482,7 +24057,7 @@
         <v>0.49</v>
       </c>
       <c r="G33" s="3">
-        <f>(C33-B33)</f>
+        <f t="shared" si="0"/>
         <v>263</v>
       </c>
       <c r="H33" t="str" cm="1">
@@ -23508,7 +24083,7 @@
         <v>0.49</v>
       </c>
       <c r="G34" s="3">
-        <f>(C34-B34)</f>
+        <f t="shared" ref="G34:G65" si="1">(C34-B34)</f>
         <v>169</v>
       </c>
       <c r="H34" t="str" cm="1">
@@ -23540,7 +24115,7 @@
         <v>4.3</v>
       </c>
       <c r="G35" s="3">
-        <f>(C35-B35)</f>
+        <f t="shared" si="1"/>
         <v>1670</v>
       </c>
       <c r="H35" t="str" cm="1">
@@ -23566,7 +24141,7 @@
         <v>0.48</v>
       </c>
       <c r="G36" s="3">
-        <f>(C36-B36)</f>
+        <f t="shared" si="1"/>
         <v>644</v>
       </c>
       <c r="H36" t="str" cm="1">
@@ -23592,7 +24167,7 @@
         <v>0.48</v>
       </c>
       <c r="G37" s="3">
-        <f>(C37-B37)</f>
+        <f t="shared" si="1"/>
         <v>1200</v>
       </c>
       <c r="H37" t="str" cm="1">
@@ -23618,7 +24193,7 @@
         <v>0.48</v>
       </c>
       <c r="G38" s="3">
-        <f>(C38-B38)</f>
+        <f t="shared" si="1"/>
         <v>95</v>
       </c>
       <c r="H38" t="str" cm="1">
@@ -23650,7 +24225,7 @@
         <v>2.1</v>
       </c>
       <c r="G39" s="3">
-        <f>(C39-B39)</f>
+        <f t="shared" si="1"/>
         <v>1418</v>
       </c>
       <c r="H39" t="str" cm="1">
@@ -23661,8 +24236,8 @@
         <f t="array" ref="I39">_xlfn.IFS(D38&lt;=20%,"Low Disount",D38&lt;=40%,"Medium Discount",D38&gt;40%,"High Discount")</f>
         <v>High Discount</v>
       </c>
-      <c r="K39" s="14"/>
-      <c r="L39" s="14"/>
+      <c r="K39" s="13"/>
+      <c r="L39" s="13"/>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
@@ -23684,7 +24259,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="G40" s="3">
-        <f>(C40-B40)</f>
+        <f t="shared" si="1"/>
         <v>846</v>
       </c>
       <c r="H40" t="str" cm="1">
@@ -23695,8 +24270,8 @@
         <f t="array" ref="I40">_xlfn.IFS(D39&lt;=20%,"Low Disount",D39&lt;=40%,"Medium Discount",D39&gt;40%,"High Discount")</f>
         <v>High Discount</v>
       </c>
-      <c r="K40" s="14"/>
-      <c r="L40" s="14"/>
+      <c r="K40" s="13"/>
+      <c r="L40" s="13"/>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
@@ -23718,7 +24293,7 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="G41" s="3">
-        <f>(C41-B41)</f>
+        <f t="shared" si="1"/>
         <v>472</v>
       </c>
       <c r="H41" t="str" cm="1">
@@ -23750,7 +24325,7 @@
         <v>4.8</v>
       </c>
       <c r="G42" s="3">
-        <f>(C42-B42)</f>
+        <f t="shared" si="1"/>
         <v>483</v>
       </c>
       <c r="H42" t="str" cm="1">
@@ -23776,7 +24351,7 @@
         <v>0.47</v>
       </c>
       <c r="G43" s="3">
-        <f>(C43-B43)</f>
+        <f t="shared" si="1"/>
         <v>695</v>
       </c>
       <c r="H43" t="str" cm="1">
@@ -23802,7 +24377,7 @@
         <v>0.47</v>
       </c>
       <c r="G44" s="3">
-        <f>(C44-B44)</f>
+        <f t="shared" si="1"/>
         <v>800</v>
       </c>
       <c r="H44" t="str" cm="1">
@@ -23828,7 +24403,7 @@
         <v>0.47</v>
       </c>
       <c r="G45" s="3">
-        <f>(C45-B45)</f>
+        <f t="shared" si="1"/>
         <v>151</v>
       </c>
       <c r="H45" t="str" cm="1">
@@ -23860,7 +24435,7 @@
         <v>3</v>
       </c>
       <c r="G46" s="3">
-        <f>(C46-B46)</f>
+        <f t="shared" si="1"/>
         <v>1010</v>
       </c>
       <c r="H46" t="str" cm="1">
@@ -23892,7 +24467,7 @@
         <v>5</v>
       </c>
       <c r="G47" s="3">
-        <f>(C47-B47)</f>
+        <f t="shared" si="1"/>
         <v>165</v>
       </c>
       <c r="H47" t="str" cm="1">
@@ -23918,7 +24493,7 @@
         <v>0.46</v>
       </c>
       <c r="G48" s="3">
-        <f>(C48-B48)</f>
+        <f t="shared" si="1"/>
         <v>1880</v>
       </c>
       <c r="H48" t="str" cm="1">
@@ -23950,7 +24525,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="G49" s="3">
-        <f>(C49-B49)</f>
+        <f t="shared" si="1"/>
         <v>824</v>
       </c>
       <c r="H49" t="str" cm="1">
@@ -23961,8 +24536,8 @@
         <f t="array" ref="I49">_xlfn.IFS(D48&lt;=20%,"Low Disount",D48&lt;=40%,"Medium Discount",D48&gt;40%,"High Discount")</f>
         <v>High Discount</v>
       </c>
-      <c r="K49" s="14"/>
-      <c r="L49" s="14"/>
+      <c r="K49" s="13"/>
+      <c r="L49" s="13"/>
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
@@ -23984,7 +24559,7 @@
         <v>2.6</v>
       </c>
       <c r="G50" s="3">
-        <f>(C50-B50)</f>
+        <f t="shared" si="1"/>
         <v>318</v>
       </c>
       <c r="H50" t="str" cm="1">
@@ -24016,7 +24591,7 @@
         <v>3.8</v>
       </c>
       <c r="G51" s="3">
-        <f>(C51-B51)</f>
+        <f t="shared" si="1"/>
         <v>1329</v>
       </c>
       <c r="H51" t="str" cm="1">
@@ -24042,7 +24617,7 @@
         <v>0.45</v>
       </c>
       <c r="G52" s="3">
-        <f>(C52-B52)</f>
+        <f t="shared" si="1"/>
         <v>401</v>
       </c>
       <c r="H52" t="str" cm="1">
@@ -24074,7 +24649,7 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="G53" s="3">
-        <f>(C53-B53)</f>
+        <f t="shared" si="1"/>
         <v>257</v>
       </c>
       <c r="H53" t="str" cm="1">
@@ -24085,8 +24660,8 @@
         <f t="array" ref="I53">_xlfn.IFS(D52&lt;=20%,"Low Disount",D52&lt;=40%,"Medium Discount",D52&gt;40%,"High Discount")</f>
         <v>High Discount</v>
       </c>
-      <c r="K53" s="14"/>
-      <c r="L53" s="14"/>
+      <c r="K53" s="13"/>
+      <c r="L53" s="13"/>
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
@@ -24108,7 +24683,7 @@
         <v>3</v>
       </c>
       <c r="G54" s="3">
-        <f>(C54-B54)</f>
+        <f t="shared" si="1"/>
         <v>390</v>
       </c>
       <c r="H54" t="str" cm="1">
@@ -24134,7 +24709,7 @@
         <v>0.43</v>
       </c>
       <c r="G55" s="3">
-        <f>(C55-B55)</f>
+        <f t="shared" si="1"/>
         <v>510</v>
       </c>
       <c r="H55" t="str" cm="1">
@@ -24160,7 +24735,7 @@
         <v>0.43</v>
       </c>
       <c r="G56" s="3">
-        <f>(C56-B56)</f>
+        <f t="shared" si="1"/>
         <v>470</v>
       </c>
       <c r="H56" t="str" cm="1">
@@ -24192,7 +24767,7 @@
         <v>4.5</v>
       </c>
       <c r="G57" s="3">
-        <f>(C57-B57)</f>
+        <f t="shared" si="1"/>
         <v>359</v>
       </c>
       <c r="H57" t="str" cm="1">
@@ -24218,7 +24793,7 @@
         <v>0.42</v>
       </c>
       <c r="G58" s="3">
-        <f>(C58-B58)</f>
+        <f t="shared" si="1"/>
         <v>1360</v>
       </c>
       <c r="H58" t="str" cm="1">
@@ -24244,7 +24819,7 @@
         <v>0.42</v>
       </c>
       <c r="G59" s="3">
-        <f>(C59-B59)</f>
+        <f t="shared" si="1"/>
         <v>794</v>
       </c>
       <c r="H59" t="str" cm="1">
@@ -24270,7 +24845,7 @@
         <v>0.42</v>
       </c>
       <c r="G60" s="3">
-        <f>(C60-B60)</f>
+        <f t="shared" si="1"/>
         <v>450</v>
       </c>
       <c r="H60" t="str" cm="1">
@@ -24302,7 +24877,7 @@
         <v>4.3</v>
       </c>
       <c r="G61" s="3">
-        <f>(C61-B61)</f>
+        <f t="shared" si="1"/>
         <v>267</v>
       </c>
       <c r="H61" t="str" cm="1">
@@ -24328,7 +24903,7 @@
         <v>0.41</v>
       </c>
       <c r="G62" s="3">
-        <f>(C62-B62)</f>
+        <f t="shared" si="1"/>
         <v>1000</v>
       </c>
       <c r="H62" t="str" cm="1">
@@ -24354,7 +24929,7 @@
         <v>0.41</v>
       </c>
       <c r="G63" s="3">
-        <f>(C63-B63)</f>
+        <f t="shared" si="1"/>
         <v>544</v>
       </c>
       <c r="H63" t="str" cm="1">
@@ -24386,7 +24961,7 @@
         <v>5</v>
       </c>
       <c r="G64" s="3">
-        <f>(C64-B64)</f>
+        <f t="shared" si="1"/>
         <v>1070</v>
       </c>
       <c r="H64" t="str" cm="1">
@@ -24418,7 +24993,7 @@
         <v>3</v>
       </c>
       <c r="G65" s="3">
-        <f>(C65-B65)</f>
+        <f t="shared" si="1"/>
         <v>2393</v>
       </c>
       <c r="H65" t="str" cm="1">
@@ -24450,7 +25025,7 @@
         <v>4.5</v>
       </c>
       <c r="G66" s="3">
-        <f>(C66-B66)</f>
+        <f t="shared" ref="G66:G97" si="2">(C66-B66)</f>
         <v>900</v>
       </c>
       <c r="H66" t="str" cm="1">
@@ -24482,7 +25057,7 @@
         <v>4.5</v>
       </c>
       <c r="G67" s="3">
-        <f>(C67-B67)</f>
+        <f t="shared" si="2"/>
         <v>575</v>
       </c>
       <c r="H67" t="str" cm="1">
@@ -24508,7 +25083,7 @@
         <v>0.38</v>
       </c>
       <c r="G68" s="3">
-        <f>(C68-B68)</f>
+        <f t="shared" si="2"/>
         <v>750</v>
       </c>
       <c r="H68" t="str" cm="1">
@@ -24534,7 +25109,7 @@
         <v>0.38</v>
       </c>
       <c r="G69" s="3">
-        <f>(C69-B69)</f>
+        <f t="shared" si="2"/>
         <v>1721</v>
       </c>
       <c r="H69" t="str" cm="1">
@@ -24566,7 +25141,7 @@
         <v>4</v>
       </c>
       <c r="G70" s="3">
-        <f>(C70-B70)</f>
+        <f t="shared" si="2"/>
         <v>592</v>
       </c>
       <c r="H70" t="str" cm="1">
@@ -24598,7 +25173,7 @@
         <v>4.7</v>
       </c>
       <c r="G71" s="3">
-        <f>(C71-B71)</f>
+        <f t="shared" si="2"/>
         <v>919</v>
       </c>
       <c r="H71" t="str" cm="1">
@@ -24624,7 +25199,7 @@
         <v>0.36</v>
       </c>
       <c r="G72" s="3">
-        <f>(C72-B72)</f>
+        <f t="shared" si="2"/>
         <v>830</v>
       </c>
       <c r="H72" t="str" cm="1">
@@ -24656,7 +25231,7 @@
         <v>4</v>
       </c>
       <c r="G73" s="3">
-        <f>(C73-B73)</f>
+        <f t="shared" si="2"/>
         <v>470</v>
       </c>
       <c r="H73" t="str" cm="1">
@@ -24688,7 +25263,7 @@
         <v>4.5999999999999996</v>
       </c>
       <c r="G74" s="3">
-        <f>(C74-B74)</f>
+        <f t="shared" si="2"/>
         <v>227</v>
       </c>
       <c r="H74" t="str" cm="1">
@@ -24720,7 +25295,7 @@
         <v>4.7</v>
       </c>
       <c r="G75" s="3">
-        <f>(C75-B75)</f>
+        <f t="shared" si="2"/>
         <v>510</v>
       </c>
       <c r="H75" t="str" cm="1">
@@ -24752,7 +25327,7 @@
         <v>4.7</v>
       </c>
       <c r="G76" s="3">
-        <f>(C76-B76)</f>
+        <f t="shared" si="2"/>
         <v>510</v>
       </c>
       <c r="H76" t="str" cm="1">
@@ -24778,7 +25353,7 @@
         <v>0.34</v>
       </c>
       <c r="G77" s="3">
-        <f>(C77-B77)</f>
+        <f t="shared" si="2"/>
         <v>620</v>
       </c>
       <c r="H77" t="str" cm="1">
@@ -24804,7 +25379,7 @@
         <v>0.34</v>
       </c>
       <c r="G78" s="3">
-        <f>(C78-B78)</f>
+        <f t="shared" si="2"/>
         <v>587</v>
       </c>
       <c r="H78" t="str" cm="1">
@@ -24836,7 +25411,7 @@
         <v>4.2</v>
       </c>
       <c r="G79" s="3">
-        <f>(C79-B79)</f>
+        <f t="shared" si="2"/>
         <v>819</v>
       </c>
       <c r="H79" t="str" cm="1">
@@ -24862,7 +25437,7 @@
         <v>0.33</v>
       </c>
       <c r="G80" s="3">
-        <f>(C80-B80)</f>
+        <f t="shared" si="2"/>
         <v>595</v>
       </c>
       <c r="H80" t="str" cm="1">
@@ -24894,7 +25469,7 @@
         <v>3.8</v>
       </c>
       <c r="G81" s="3">
-        <f>(C81-B81)</f>
+        <f t="shared" si="2"/>
         <v>640</v>
       </c>
       <c r="H81" t="str" cm="1">
@@ -24926,7 +25501,7 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="G82" s="3">
-        <f>(C82-B82)</f>
+        <f t="shared" si="2"/>
         <v>741</v>
       </c>
       <c r="H82" t="str" cm="1">
@@ -24958,7 +25533,7 @@
         <v>3</v>
       </c>
       <c r="G83" s="3">
-        <f>(C83-B83)</f>
+        <f t="shared" si="2"/>
         <v>940</v>
       </c>
       <c r="H83" t="str" cm="1">
@@ -24990,7 +25565,7 @@
         <v>4.5</v>
       </c>
       <c r="G84" s="3">
-        <f>(C84-B84)</f>
+        <f t="shared" si="2"/>
         <v>719</v>
       </c>
       <c r="H84" t="str" cm="1">
@@ -25022,7 +25597,7 @@
         <v>4.7</v>
       </c>
       <c r="G85" s="3">
-        <f>(C85-B85)</f>
+        <f t="shared" si="2"/>
         <v>710</v>
       </c>
       <c r="H85" t="str" cm="1">
@@ -25048,7 +25623,7 @@
         <v>0.27</v>
       </c>
       <c r="G86" s="3">
-        <f>(C86-B86)</f>
+        <f t="shared" si="2"/>
         <v>1011</v>
       </c>
       <c r="H86" t="str" cm="1">
@@ -25080,7 +25655,7 @@
         <v>4.8</v>
       </c>
       <c r="G87" s="3">
-        <f>(C87-B87)</f>
+        <f t="shared" si="2"/>
         <v>616</v>
       </c>
       <c r="H87" t="str" cm="1">
@@ -25112,7 +25687,7 @@
         <v>4.5999999999999996</v>
       </c>
       <c r="G88" s="3">
-        <f>(C88-B88)</f>
+        <f t="shared" si="2"/>
         <v>724</v>
       </c>
       <c r="H88" t="str" cm="1">
@@ -25144,7 +25719,7 @@
         <v>4.5999999999999996</v>
       </c>
       <c r="G89" s="3">
-        <f>(C89-B89)</f>
+        <f t="shared" si="2"/>
         <v>713</v>
       </c>
       <c r="H89" t="str" cm="1">
@@ -25170,7 +25745,7 @@
         <v>0.24</v>
       </c>
       <c r="G90" s="3">
-        <f>(C90-B90)</f>
+        <f t="shared" si="2"/>
         <v>62</v>
       </c>
       <c r="H90" t="str" cm="1">
@@ -25202,7 +25777,7 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="G91" s="3">
-        <f>(C91-B91)</f>
+        <f t="shared" si="2"/>
         <v>500</v>
       </c>
       <c r="H91" t="str" cm="1">
@@ -25234,7 +25809,7 @@
         <v>2.9</v>
       </c>
       <c r="G92" s="3">
-        <f>(C92-B92)</f>
+        <f t="shared" si="2"/>
         <v>335</v>
       </c>
       <c r="H92" t="str" cm="1">
@@ -25260,7 +25835,7 @@
         <v>0.22</v>
       </c>
       <c r="G93" s="3">
-        <f>(C93-B93)</f>
+        <f t="shared" si="2"/>
         <v>85</v>
       </c>
       <c r="H93" t="str" cm="1">
@@ -25292,7 +25867,7 @@
         <v>5</v>
       </c>
       <c r="G94" s="3">
-        <f>(C94-B94)</f>
+        <f t="shared" si="2"/>
         <v>948</v>
       </c>
       <c r="H94" t="str" cm="1">
@@ -25324,7 +25899,7 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="G95" s="3">
-        <f>(C95-B95)</f>
+        <f t="shared" si="2"/>
         <v>200</v>
       </c>
       <c r="H95" t="str" cm="1">
@@ -25356,7 +25931,7 @@
         <v>4.5999999999999996</v>
       </c>
       <c r="G96" s="3">
-        <f>(C96-B96)</f>
+        <f t="shared" si="2"/>
         <v>700</v>
       </c>
       <c r="H96" t="str" cm="1">
@@ -25388,7 +25963,7 @@
         <v>3.8</v>
       </c>
       <c r="G97" s="3">
-        <f>(C97-B97)</f>
+        <f t="shared" si="2"/>
         <v>640</v>
       </c>
       <c r="H97" t="str" cm="1">
@@ -25414,7 +25989,7 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="G98" s="3">
-        <f>(C98-B98)</f>
+        <f t="shared" ref="G98:G113" si="3">(C98-B98)</f>
         <v>233</v>
       </c>
       <c r="H98" t="str" cm="1">
@@ -25440,7 +26015,7 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="G99" s="3">
-        <f>(C99-B99)</f>
+        <f t="shared" si="3"/>
         <v>231</v>
       </c>
       <c r="H99" t="str" cm="1">
@@ -25472,7 +26047,7 @@
         <v>2.5</v>
       </c>
       <c r="G100" s="3">
-        <f>(C100-B100)</f>
+        <f t="shared" si="3"/>
         <v>330</v>
       </c>
       <c r="H100" t="str" cm="1">
@@ -25498,7 +26073,7 @@
         <v>0.11</v>
       </c>
       <c r="G101" s="3">
-        <f>(C101-B101)</f>
+        <f t="shared" si="3"/>
         <v>101</v>
       </c>
       <c r="H101" t="str" cm="1">
@@ -25530,7 +26105,7 @@
         <v>4</v>
       </c>
       <c r="G102" s="3">
-        <f>(C102-B102)</f>
+        <f t="shared" si="3"/>
         <v>291</v>
       </c>
       <c r="H102" t="str" cm="1">
@@ -25556,7 +26131,7 @@
         <v>0.08</v>
       </c>
       <c r="G103" s="3">
-        <f>(C103-B103)</f>
+        <f t="shared" si="3"/>
         <v>134</v>
       </c>
       <c r="H103" t="str" cm="1">
@@ -25582,7 +26157,7 @@
         <v>0.04</v>
       </c>
       <c r="G104" s="3">
-        <f>(C104-B104)</f>
+        <f t="shared" si="3"/>
         <v>67</v>
       </c>
       <c r="H104" t="str" cm="1">
@@ -25608,7 +26183,7 @@
         <v>0.04</v>
       </c>
       <c r="G105" s="3">
-        <f>(C105-B105)</f>
+        <f t="shared" si="3"/>
         <v>153</v>
       </c>
       <c r="H105" t="str" cm="1">
@@ -25634,7 +26209,7 @@
         <v>0.03</v>
       </c>
       <c r="G106" s="3">
-        <f>(C106-B106)</f>
+        <f t="shared" si="3"/>
         <v>40</v>
       </c>
       <c r="H106" t="str" cm="1">
@@ -25660,7 +26235,7 @@
         <v>0.02</v>
       </c>
       <c r="G107" s="3">
-        <f>(C107-B107)</f>
+        <f t="shared" si="3"/>
         <v>33</v>
       </c>
       <c r="H107" t="str" cm="1">
@@ -25686,7 +26261,7 @@
         <v>0.02</v>
       </c>
       <c r="G108" s="3">
-        <f>(C108-B108)</f>
+        <f t="shared" si="3"/>
         <v>39</v>
       </c>
       <c r="H108" t="str" cm="1">
@@ -25712,7 +26287,7 @@
         <v>0.02</v>
       </c>
       <c r="G109" s="3">
-        <f>(C109-B109)</f>
+        <f t="shared" si="3"/>
         <v>37</v>
       </c>
       <c r="H109" t="str" cm="1">
@@ -25738,7 +26313,7 @@
         <v>0.02</v>
       </c>
       <c r="G110" s="3">
-        <f>(C110-B110)</f>
+        <f t="shared" si="3"/>
         <v>37</v>
       </c>
       <c r="H110" t="str" cm="1">
@@ -25764,7 +26339,7 @@
         <v>0.02</v>
       </c>
       <c r="G111" s="3">
-        <f>(C111-B111)</f>
+        <f t="shared" si="3"/>
         <v>41</v>
       </c>
       <c r="H111" t="str" cm="1">
@@ -25790,7 +26365,7 @@
         <v>0.02</v>
       </c>
       <c r="G112" s="3">
-        <f>(C112-B112)</f>
+        <f t="shared" si="3"/>
         <v>31</v>
       </c>
       <c r="H112" t="str" cm="1">
@@ -25816,7 +26391,7 @@
         <v>0.01</v>
       </c>
       <c r="G113" s="3">
-        <f>(C113-B113)</f>
+        <f t="shared" si="3"/>
         <v>24</v>
       </c>
       <c r="H113" t="str" cm="1">
@@ -25836,7 +26411,7 @@
     <sortCondition descending="1" ref="D1:D113"/>
   </sortState>
   <conditionalFormatting sqref="D1:D1048576">
-    <cfRule type="top10" dxfId="0" priority="1" rank="10"/>
+    <cfRule type="top10" dxfId="4" priority="1" rank="10"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -25867,7 +26442,7 @@
       <c r="A4" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="17">
         <v>15</v>
       </c>
     </row>
@@ -25875,7 +26450,7 @@
       <c r="A5" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="17">
         <v>35</v>
       </c>
     </row>
@@ -25883,7 +26458,7 @@
       <c r="A6" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="B6" s="13">
+      <c r="B6" s="17">
         <v>192</v>
       </c>
     </row>
@@ -25891,7 +26466,7 @@
       <c r="A7" s="11" t="s">
         <v>129</v>
       </c>
-      <c r="B7" s="13">
+      <c r="B7" s="17">
         <v>147</v>
       </c>
     </row>
@@ -25899,7 +26474,7 @@
       <c r="A8" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="B8" s="13">
+      <c r="B8" s="17">
         <v>258</v>
       </c>
     </row>
@@ -25907,7 +26482,7 @@
       <c r="A9" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="B9" s="13">
+      <c r="B9" s="17">
         <v>76</v>
       </c>
     </row>
@@ -25915,13 +26490,13 @@
       <c r="A10" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="B10" s="13"/>
+      <c r="B10" s="17"/>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="B11" s="13">
+      <c r="B11" s="17">
         <v>723</v>
       </c>
     </row>
@@ -25959,7 +26534,7 @@
       <c r="A4" s="10">
         <v>2</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="17">
         <v>1</v>
       </c>
     </row>
@@ -25967,7 +26542,7 @@
       <c r="A5" s="10">
         <v>2.1</v>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="17">
         <v>20</v>
       </c>
     </row>
@@ -25975,7 +26550,7 @@
       <c r="A6" s="10">
         <v>2.2000000000000002</v>
       </c>
-      <c r="B6" s="13">
+      <c r="B6" s="17">
         <v>12</v>
       </c>
     </row>
@@ -25983,7 +26558,7 @@
       <c r="A7" s="10">
         <v>2.2999999999999998</v>
       </c>
-      <c r="B7" s="13">
+      <c r="B7" s="17">
         <v>13</v>
       </c>
     </row>
@@ -25991,7 +26566,7 @@
       <c r="A8" s="10">
         <v>2.5</v>
       </c>
-      <c r="B8" s="13">
+      <c r="B8" s="17">
         <v>6</v>
       </c>
     </row>
@@ -25999,7 +26574,7 @@
       <c r="A9" s="10">
         <v>2.6</v>
       </c>
-      <c r="B9" s="13">
+      <c r="B9" s="17">
         <v>17</v>
       </c>
     </row>
@@ -26007,7 +26582,7 @@
       <c r="A10" s="10">
         <v>2.7</v>
       </c>
-      <c r="B10" s="13">
+      <c r="B10" s="17">
         <v>15</v>
       </c>
     </row>
@@ -26015,7 +26590,7 @@
       <c r="A11" s="10">
         <v>2.8</v>
       </c>
-      <c r="B11" s="13">
+      <c r="B11" s="17">
         <v>69</v>
       </c>
     </row>
@@ -26023,7 +26598,7 @@
       <c r="A12" s="10">
         <v>2.9</v>
       </c>
-      <c r="B12" s="13">
+      <c r="B12" s="17">
         <v>16</v>
       </c>
     </row>
@@ -26031,7 +26606,7 @@
       <c r="A13" s="10">
         <v>3</v>
       </c>
-      <c r="B13" s="13">
+      <c r="B13" s="17">
         <v>26</v>
       </c>
     </row>
@@ -26039,7 +26614,7 @@
       <c r="A14" s="10">
         <v>3.3</v>
       </c>
-      <c r="B14" s="13">
+      <c r="B14" s="17">
         <v>13</v>
       </c>
     </row>
@@ -26047,7 +26622,7 @@
       <c r="A15" s="10">
         <v>3.8</v>
       </c>
-      <c r="B15" s="13">
+      <c r="B15" s="17">
         <v>30</v>
       </c>
     </row>
@@ -26055,7 +26630,7 @@
       <c r="A16" s="10">
         <v>4</v>
       </c>
-      <c r="B16" s="13">
+      <c r="B16" s="17">
         <v>24</v>
       </c>
     </row>
@@ -26063,7 +26638,7 @@
       <c r="A17" s="10">
         <v>4.0999999999999996</v>
       </c>
-      <c r="B17" s="13">
+      <c r="B17" s="17">
         <v>46</v>
       </c>
     </row>
@@ -26071,7 +26646,7 @@
       <c r="A18" s="10">
         <v>4.2</v>
       </c>
-      <c r="B18" s="13">
+      <c r="B18" s="17">
         <v>9</v>
       </c>
     </row>
@@ -26079,7 +26654,7 @@
       <c r="A19" s="10">
         <v>4.3</v>
       </c>
-      <c r="B19" s="13">
+      <c r="B19" s="17">
         <v>61</v>
       </c>
     </row>
@@ -26087,7 +26662,7 @@
       <c r="A20" s="10">
         <v>4.4000000000000004</v>
       </c>
-      <c r="B20" s="13">
+      <c r="B20" s="17">
         <v>14</v>
       </c>
     </row>
@@ -26095,7 +26670,7 @@
       <c r="A21" s="10">
         <v>4.5</v>
       </c>
-      <c r="B21" s="13">
+      <c r="B21" s="17">
         <v>42</v>
       </c>
     </row>
@@ -26103,7 +26678,7 @@
       <c r="A22" s="10">
         <v>4.5999999999999996</v>
       </c>
-      <c r="B22" s="13">
+      <c r="B22" s="17">
         <v>177</v>
       </c>
     </row>
@@ -26111,7 +26686,7 @@
       <c r="A23" s="10">
         <v>4.7</v>
       </c>
-      <c r="B23" s="13">
+      <c r="B23" s="17">
         <v>78</v>
       </c>
     </row>
@@ -26119,7 +26694,7 @@
       <c r="A24" s="10">
         <v>4.8</v>
       </c>
-      <c r="B24" s="13">
+      <c r="B24" s="17">
         <v>22</v>
       </c>
     </row>
@@ -26127,7 +26702,7 @@
       <c r="A25" s="10">
         <v>5</v>
       </c>
-      <c r="B25" s="13">
+      <c r="B25" s="17">
         <v>12</v>
       </c>
     </row>
@@ -26135,13 +26710,13 @@
       <c r="A26" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="B26" s="13"/>
+      <c r="B26" s="17"/>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="B27" s="13">
+      <c r="B27" s="17">
         <v>723</v>
       </c>
     </row>
@@ -26187,7 +26762,7 @@
       <c r="A4" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="17">
         <v>5</v>
       </c>
     </row>
@@ -26195,7 +26770,7 @@
       <c r="A5" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="17">
         <v>5</v>
       </c>
     </row>
@@ -26203,7 +26778,7 @@
       <c r="A6" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="13">
+      <c r="B6" s="17">
         <v>5</v>
       </c>
     </row>
@@ -26211,7 +26786,7 @@
       <c r="A7" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="B7" s="13">
+      <c r="B7" s="17">
         <v>5</v>
       </c>
     </row>
@@ -26219,7 +26794,7 @@
       <c r="A8" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="B8" s="13">
+      <c r="B8" s="17">
         <v>5</v>
       </c>
     </row>
@@ -26227,7 +26802,7 @@
       <c r="A9" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="13">
+      <c r="B9" s="17">
         <v>5</v>
       </c>
     </row>
@@ -26235,7 +26810,7 @@
       <c r="A10" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="13">
+      <c r="B10" s="17">
         <v>5</v>
       </c>
     </row>
@@ -26243,7 +26818,7 @@
       <c r="A11" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="B11" s="13">
+      <c r="B11" s="17">
         <v>35</v>
       </c>
     </row>
@@ -26254,11 +26829,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{848CDC0A-84C5-4D71-9474-81BA0596BF0B}">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B113"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="63.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="85.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -26266,7 +26841,7 @@
         <v>5</v>
       </c>
       <c r="B1" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -26279,50 +26854,778 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="B4" s="13">
-        <v>2</v>
-      </c>
+        <v>81</v>
+      </c>
+      <c r="B4" s="17"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="B5" s="13">
-        <v>2.1</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="B5" s="17"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="B6" s="13">
-        <v>2.1</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="B6" s="17"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="B7" s="13">
-        <v>2.2000000000000002</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="B7" s="17"/>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="B8" s="13">
-        <v>2.2000000000000002</v>
-      </c>
+        <v>63</v>
+      </c>
+      <c r="B8" s="17"/>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="B9" s="17"/>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="B10" s="17"/>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="B11" s="17"/>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="B12" s="17"/>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B13" s="17"/>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B14" s="17"/>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="B15" s="17"/>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="B16" s="17"/>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B17" s="17"/>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="B18" s="17"/>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="B19" s="17"/>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="B20" s="17"/>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="B21" s="17"/>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="B22" s="17"/>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="B23" s="17"/>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="B24" s="17"/>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="B25" s="17"/>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="B26" s="17"/>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="B27" s="17"/>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="B28" s="17"/>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B29" s="17"/>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="B30" s="17"/>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B31" s="17"/>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="B32" s="17"/>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="B33" s="17"/>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="B34" s="17"/>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="B35" s="17"/>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="B36" s="17"/>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A37" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B37" s="17"/>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A38" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="B38" s="17"/>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A39" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="B39" s="17"/>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A40" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="B40" s="17"/>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A41" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="B41" s="17"/>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A42" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="B42" s="17"/>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A43" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="B43" s="17"/>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A44" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="B44" s="17"/>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A45" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="B45" s="17"/>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A46" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B46" s="17"/>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A47" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="B47" s="17"/>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A48" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="B48" s="17"/>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="B49" s="17"/>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="B50" s="17"/>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A51" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="B51" s="17"/>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="B52" s="17"/>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A53" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="B53" s="17"/>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A54" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="B54" s="17"/>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A55" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="B55" s="17"/>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A56" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="B56" s="17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A57" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="B57" s="17">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A58" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="B58" s="17">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A59" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="B59" s="17">
+        <v>2.2000000000000002</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A60" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="B60" s="17">
+        <v>2.2000000000000002</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A61" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="B61" s="17">
+        <v>2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A62" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="B62" s="17">
+        <v>2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A63" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="B63" s="17">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A64" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="B64" s="17">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A65" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B65" s="17">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A66" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="B66" s="17">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A67" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="B67" s="17">
+        <v>2.9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A68" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="B68" s="17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A69" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B69" s="17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A70" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B70" s="17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A71" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="B71" s="17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A72" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="B72" s="17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A73" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B73" s="17">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A74" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B74" s="17">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A75" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B75" s="17">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A76" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B76" s="17">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A77" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B77" s="17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A78" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B78" s="17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A79" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="B79" s="17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A80" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B80" s="17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A81" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B81" s="17">
+        <v>4.0999999999999996</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A82" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B82" s="17">
+        <v>4.0999999999999996</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A83" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B83" s="17">
+        <v>4.0999999999999996</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A84" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B84" s="17">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A85" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="B85" s="17">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A86" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="B86" s="17">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A87" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B87" s="17">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A88" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B88" s="17">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A89" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B89" s="17">
+        <v>4.4000000000000004</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A90" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B90" s="17">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A91" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B91" s="17">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A92" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B92" s="17">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A93" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="B93" s="17">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A94" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B94" s="17">
+        <v>4.5999999999999996</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A95" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B95" s="17">
+        <v>4.5999999999999996</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A96" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B96" s="17">
+        <v>4.5999999999999996</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A97" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B97" s="17">
+        <v>4.5999999999999996</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A98" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B98" s="17">
+        <v>4.5999999999999996</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A99" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B99" s="17">
+        <v>4.7</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A100" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B100" s="17">
+        <v>4.7</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A101" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B101" s="17">
+        <v>4.7</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A102" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B102" s="17">
+        <v>4.7</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A103" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B103" s="17">
+        <v>4.8</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A104" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B104" s="17">
+        <v>4.8</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A105" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B105" s="17">
+        <v>4.8</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A106" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B106" s="17">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A107" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B107" s="17">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A108" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B108" s="17">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A109" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="B109" s="17">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A110" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B110" s="17">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A111" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="B111" s="17">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A112" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B112" s="17">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A113" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="B9" s="13">
-        <v>10.600000000000001</v>
+      <c r="B113" s="17">
+        <v>221.70000000000002</v>
       </c>
     </row>
   </sheetData>
@@ -26345,42 +27648,42 @@
         <v>122</v>
       </c>
       <c r="B3" t="s">
+        <v>138</v>
+      </c>
+      <c r="C3" t="s">
         <v>139</v>
-      </c>
-      <c r="C3" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
-        <v>136</v>
-      </c>
-      <c r="B4" s="13">
+        <v>135</v>
+      </c>
+      <c r="B4" s="17">
         <v>3.5766666666666658</v>
       </c>
-      <c r="C4" s="13">
+      <c r="C4" s="17">
         <v>13.533333333333333</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>137</v>
-      </c>
-      <c r="B5" s="13">
+        <v>136</v>
+      </c>
+      <c r="B5" s="17">
         <v>3.8599999999999994</v>
       </c>
-      <c r="C5" s="13">
+      <c r="C5" s="17">
         <v>14.4</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
-        <v>138</v>
-      </c>
-      <c r="B6" s="13">
+        <v>137</v>
+      </c>
+      <c r="B6" s="17">
         <v>4.3142857142857149</v>
       </c>
-      <c r="C6" s="13">
+      <c r="C6" s="17">
         <v>11.571428571428571</v>
       </c>
     </row>
@@ -26388,10 +27691,10 @@
       <c r="A7" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="B7" s="13">
+      <c r="B7" s="17">
         <v>4.5</v>
       </c>
-      <c r="C7" s="13">
+      <c r="C7" s="17">
         <v>2</v>
       </c>
     </row>
@@ -26399,10 +27702,10 @@
       <c r="A8" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="B8" s="13">
+      <c r="B8" s="17">
         <v>3.8894736842105253</v>
       </c>
-      <c r="C8" s="13">
+      <c r="C8" s="17">
         <v>12.684210526315789</v>
       </c>
     </row>
@@ -26445,17 +27748,17 @@
         <v>134</v>
       </c>
       <c r="D3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B4">
         <v>39</v>
       </c>
-      <c r="C4" s="13">
+      <c r="C4">
         <v>4.7</v>
       </c>
       <c r="D4" s="1">
@@ -26466,10 +27769,10 @@
       <c r="A5" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="B5" s="13">
+      <c r="B5">
         <v>69</v>
       </c>
-      <c r="C5" s="13">
+      <c r="C5">
         <v>2.8</v>
       </c>
       <c r="D5" s="1">
@@ -26480,10 +27783,10 @@
       <c r="A6" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="13">
+      <c r="B6">
         <v>55</v>
       </c>
-      <c r="C6" s="13">
+      <c r="C6">
         <v>4.5999999999999996</v>
       </c>
       <c r="D6" s="1">
@@ -26494,10 +27797,10 @@
       <c r="A7" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="13">
+      <c r="B7">
         <v>44</v>
       </c>
-      <c r="C7" s="13">
+      <c r="C7">
         <v>4.5999999999999996</v>
       </c>
       <c r="D7" s="1">
@@ -26508,10 +27811,10 @@
       <c r="A8" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="B8" s="13">
+      <c r="B8">
         <v>20</v>
       </c>
-      <c r="C8" s="13">
+      <c r="C8">
         <v>4.0999999999999996</v>
       </c>
       <c r="D8" s="1">
@@ -26522,10 +27825,10 @@
       <c r="A9" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="13">
+      <c r="B9">
         <v>32</v>
       </c>
-      <c r="C9" s="13">
+      <c r="C9">
         <v>4.5</v>
       </c>
       <c r="D9" s="1">
@@ -26536,10 +27839,10 @@
       <c r="A10" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="13">
+      <c r="B10">
         <v>20</v>
       </c>
-      <c r="C10" s="13">
+      <c r="C10">
         <v>4.7</v>
       </c>
       <c r="D10" s="1">
@@ -26550,10 +27853,10 @@
       <c r="A11" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="13">
+      <c r="B11">
         <v>49</v>
       </c>
-      <c r="C11" s="13">
+      <c r="C11">
         <v>4.5999999999999996</v>
       </c>
       <c r="D11" s="1">
@@ -26564,10 +27867,10 @@
       <c r="A12" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="13">
+      <c r="B12">
         <v>24</v>
       </c>
-      <c r="C12" s="13">
+      <c r="C12">
         <v>4.5999999999999996</v>
       </c>
       <c r="D12" s="1">
@@ -26578,10 +27881,10 @@
       <c r="A13" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="B13" s="13">
+      <c r="B13">
         <v>36</v>
       </c>
-      <c r="C13" s="13">
+      <c r="C13">
         <v>4.3</v>
       </c>
       <c r="D13" s="1">
@@ -26592,10 +27895,10 @@
       <c r="A14" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="B14" s="13">
+      <c r="B14">
         <v>388</v>
       </c>
-      <c r="C14" s="13">
+      <c r="C14">
         <v>43.499999999999993</v>
       </c>
       <c r="D14" s="1">
@@ -26629,7 +27932,7 @@
       <c r="A4" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B4">
         <v>4.8</v>
       </c>
     </row>
@@ -26637,7 +27940,7 @@
       <c r="A5" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="13">
+      <c r="B5">
         <v>5</v>
       </c>
     </row>
@@ -26645,7 +27948,7 @@
       <c r="A6" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="B6" s="13">
+      <c r="B6">
         <v>5</v>
       </c>
     </row>
@@ -26653,7 +27956,7 @@
       <c r="A7" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="B7" s="13">
+      <c r="B7">
         <v>5</v>
       </c>
     </row>
@@ -26661,7 +27964,7 @@
       <c r="A8" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="13">
+      <c r="B8">
         <v>5</v>
       </c>
     </row>
@@ -26669,7 +27972,7 @@
       <c r="A9" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="B9" s="13">
+      <c r="B9">
         <v>5</v>
       </c>
     </row>
@@ -26677,7 +27980,7 @@
       <c r="A10" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="13">
+      <c r="B10">
         <v>5</v>
       </c>
     </row>
@@ -26685,7 +27988,7 @@
       <c r="A11" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="13">
+      <c r="B11">
         <v>4.8</v>
       </c>
     </row>
@@ -26693,7 +27996,7 @@
       <c r="A12" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="13">
+      <c r="B12">
         <v>5</v>
       </c>
     </row>
@@ -26701,7 +28004,7 @@
       <c r="A13" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="13">
+      <c r="B13">
         <v>4.8</v>
       </c>
     </row>
@@ -26709,7 +28012,7 @@
       <c r="A14" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="B14" s="13">
+      <c r="B14">
         <v>49.399999999999991</v>
       </c>
     </row>
@@ -26736,7 +28039,7 @@
   <sheetData>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B3" s="8" t="s">
         <v>133</v>
@@ -26747,13 +28050,13 @@
         <v>122</v>
       </c>
       <c r="B4" t="s">
+        <v>135</v>
+      </c>
+      <c r="C4" t="s">
         <v>136</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>137</v>
-      </c>
-      <c r="D4" t="s">
-        <v>138</v>
       </c>
       <c r="E4" t="s">
         <v>123</v>
@@ -26761,52 +28064,52 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>142</v>
-      </c>
-      <c r="B5" s="13">
+        <v>141</v>
+      </c>
+      <c r="B5">
         <v>5</v>
       </c>
-      <c r="C5" s="13">
+      <c r="C5">
         <v>1</v>
       </c>
-      <c r="D5" s="13">
+      <c r="D5">
         <v>3</v>
       </c>
-      <c r="E5" s="13">
+      <c r="E5">
         <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="B6" s="13">
+        <v>142</v>
+      </c>
+      <c r="B6">
         <v>16</v>
       </c>
-      <c r="C6" s="13">
+      <c r="C6">
         <v>3</v>
       </c>
-      <c r="D6" s="13">
+      <c r="D6">
         <v>18</v>
       </c>
-      <c r="E6" s="13">
+      <c r="E6">
         <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
-        <v>144</v>
-      </c>
-      <c r="B7" s="13">
+        <v>143</v>
+      </c>
+      <c r="B7">
         <v>10</v>
       </c>
-      <c r="C7" s="13">
+      <c r="C7">
         <v>1</v>
       </c>
-      <c r="D7" s="13">
+      <c r="D7">
         <v>1</v>
       </c>
-      <c r="E7" s="13">
+      <c r="E7">
         <v>12</v>
       </c>
     </row>
@@ -26814,16 +28117,16 @@
       <c r="A8" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="B8" s="13">
+      <c r="B8">
         <v>31</v>
       </c>
-      <c r="C8" s="13">
+      <c r="C8">
         <v>5</v>
       </c>
-      <c r="D8" s="13">
+      <c r="D8">
         <v>22</v>
       </c>
-      <c r="E8" s="13">
+      <c r="E8">
         <v>58</v>
       </c>
     </row>

</xml_diff>